<commit_message>
Update timeline doc file
</commit_message>
<xml_diff>
--- a/docs/Cronograma - SITUA.xlsx
+++ b/docs/Cronograma - SITUA.xlsx
@@ -22,25 +22,25 @@
     <t>Completo?</t>
   </si>
   <si>
-    <t>Sem. 1</t>
-  </si>
-  <si>
-    <t>Sem. 2</t>
-  </si>
-  <si>
-    <t>Sem. 3</t>
-  </si>
-  <si>
-    <t>Sem. 4</t>
+    <t>Sem. 1 e 2 (24/03)</t>
+  </si>
+  <si>
+    <t>Sem. 3 e 4</t>
   </si>
   <si>
     <t>Sem. 5 e 6</t>
   </si>
   <si>
-    <t>Sem. 7 e 8</t>
-  </si>
-  <si>
-    <t>Sem. 9 e 10</t>
+    <t>Sem. 7</t>
+  </si>
+  <si>
+    <t>Sem. 8</t>
+  </si>
+  <si>
+    <t>Sem. 9</t>
+  </si>
+  <si>
+    <t>Sem. 10</t>
   </si>
   <si>
     <t>Maquete - Fundamento</t>
@@ -70,25 +70,25 @@
     <t>Interface de usuário</t>
   </si>
   <si>
+    <t>Esboço</t>
+  </si>
+  <si>
+    <t>Protótipo</t>
+  </si>
+  <si>
+    <t>Melhorias e Documentação</t>
+  </si>
+  <si>
+    <t>Sensores</t>
+  </si>
+  <si>
+    <t>Posicionamento</t>
+  </si>
+  <si>
+    <t>Semáforo inteligente</t>
+  </si>
+  <si>
     <t>Média</t>
-  </si>
-  <si>
-    <t>Esboço</t>
-  </si>
-  <si>
-    <t>Protótipo</t>
-  </si>
-  <si>
-    <t>Melhorias e Documentação</t>
-  </si>
-  <si>
-    <t>Sensores</t>
-  </si>
-  <si>
-    <t>Posicionamento</t>
-  </si>
-  <si>
-    <t>Semáforo inteligente</t>
   </si>
   <si>
     <t>Placa de sinalização de trânsito</t>
@@ -296,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -305,6 +305,9 @@
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -429,13 +432,13 @@
     <tableColumn name="Parte" id="1"/>
     <tableColumn name="Prioridade" id="2"/>
     <tableColumn name="Completo?" id="3"/>
-    <tableColumn name="Sem. 1" id="4"/>
-    <tableColumn name="Sem. 2" id="5"/>
-    <tableColumn name="Sem. 3" id="6"/>
-    <tableColumn name="Sem. 4" id="7"/>
-    <tableColumn name="Sem. 5 e 6" id="8"/>
-    <tableColumn name="Sem. 7 e 8" id="9"/>
-    <tableColumn name="Sem. 9 e 10" id="10"/>
+    <tableColumn name="Sem. 1 e 2 (24/03)" id="4"/>
+    <tableColumn name="Sem. 3 e 4" id="5"/>
+    <tableColumn name="Sem. 5 e 6" id="6"/>
+    <tableColumn name="Sem. 7" id="7"/>
+    <tableColumn name="Sem. 8" id="8"/>
+    <tableColumn name="Sem. 9" id="9"/>
+    <tableColumn name="Sem. 10" id="10"/>
   </tableColumns>
   <tableStyleInfo name="Página1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -645,9 +648,9 @@
     <col customWidth="1" min="1" max="1" width="22.63"/>
     <col customWidth="1" min="2" max="2" width="16.38"/>
     <col customWidth="1" min="3" max="3" width="13.5"/>
-    <col customWidth="1" min="4" max="9" width="13.25"/>
-    <col customWidth="1" min="10" max="10" width="14.25"/>
-    <col customWidth="1" min="11" max="11" width="15.13"/>
+    <col customWidth="1" min="4" max="10" width="13.25"/>
+    <col customWidth="1" min="11" max="11" width="14.25"/>
+    <col customWidth="1" min="12" max="12" width="15.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -675,143 +678,144 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="6" t="b">
+      <c r="C2" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="8"/>
-      <c r="J2" s="7"/>
+      <c r="J2" s="8"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="11" t="b">
+      <c r="C3" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="13" t="s">
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="9"/>
+      <c r="G4" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="8"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15" t="s">
         <v>21</v>
-      </c>
-      <c r="H4" s="7"/>
-      <c r="J4" s="14" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="17"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="6" t="b">
+      <c r="C6" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="7" t="s">
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="7"/>
+      <c r="J6" s="8"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="20" t="b">
+      <c r="C7" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="21"/>
-      <c r="H7" s="22" t="s">
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="22"/>
+      <c r="H7" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
     </row>
   </sheetData>
   <dataValidations>

</xml_diff>